<commit_message>
Cierre de la Investigación Azure Machine Learning y traspaso al equipo
Fase 2/SIGMA_Investigacion_Azure_ML.docx: informe formal (objetivo, decisiones,
construido, resultados, evidencia, riesgos, recomendaciones para el Sprint 6).
MD/SIGMA_TRASPASO_EQUIPO.md: estado real de los sprints (tareas, criterios,
pruebas), qué toca a cada uno, cómo se opera SIGMA AI. Sprint Backlog S6: 7
tareas de Bryan «En revisión» y 8 anotadas como cubiertas por la investigación.
Web.config con las claves de Custom Vision (extremo público; la clave queda
en PENDIENTE en el repositorio y solo en el servidor).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S6.xlsx
+++ b/Fase 2/Sprint Backlogs/SIGMA_Sprint_Backlog_S6.xlsx
@@ -6078,6 +6078,8 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5" ht="27.75" customHeight="1" s="19">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -11752,11 +11754,17 @@
       </c>
       <c r="H139" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I139" s="11" t="n"/>
-      <c r="J139" s="12" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="I139" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J139" s="12" t="inlineStr">
+        <is>
+          <t>Investigación Azure ML: los tres modelos existen como semilla SQL (BD/245/247/248). Falta el INS_MODELO_PREDICTIVO del mantenedor.</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="55.2" customHeight="1" s="19">
       <c r="A140" s="11" t="inlineStr">
@@ -12004,11 +12012,17 @@
       </c>
       <c r="H145" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I145" s="11" t="n"/>
-      <c r="J145" s="12" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="I145" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J145" s="12" t="inlineStr">
+        <is>
+          <t>Investigación Azure ML (BD/245): menú SIGMA AI › Experimentos registrado con permiso VER PREDICCIONES.</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="27.6" customHeight="1" s="19">
       <c r="A146" s="11" t="inlineStr">
@@ -12218,7 +12232,11 @@
         </is>
       </c>
       <c r="I150" s="11" t="n"/>
-      <c r="J150" s="12" t="n"/>
+      <c r="J150" s="12" t="inlineStr">
+        <is>
+          <t>Cubierta por la investigación (mpv_parametro, mpv_registro, mpv_fecha_verificacion_utc; BD/245–246). Revisar en Sprint Planning 6.</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="41.4" customHeight="1" s="19">
       <c r="A151" s="11" t="inlineStr">
@@ -12260,7 +12278,11 @@
         </is>
       </c>
       <c r="I151" s="11" t="n"/>
-      <c r="J151" s="12" t="n"/>
+      <c r="J151" s="12" t="inlineStr">
+        <is>
+          <t>Cubierta por la investigación (API_INS_ML_ENTRENAMIENTO + API_INS_ML_MODELO_VERSION, Bryan). Revisar en Sprint Planning 6.</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="55.2" customHeight="1" s="19">
       <c r="A152" s="11" t="inlineStr">
@@ -12298,11 +12320,17 @@
       </c>
       <c r="H152" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I152" s="11" t="n"/>
-      <c r="J152" s="12" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="I152" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J152" s="12" t="inlineStr">
+        <is>
+          <t>Investigación Azure ML (BD/245–246): reglas en API_INS_ML_MODELO_VERSION (pesos válidos), API_UPD_ML_MODELO_VERSION_PUBLICAR (retira la anterior), API_UPD_ML_MODELO_VERSION_ARTEFACTO (hash del ONNX de Azure).</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="41.4" customHeight="1" s="19">
       <c r="A153" s="11" t="inlineStr">
@@ -12344,7 +12372,11 @@
         </is>
       </c>
       <c r="I153" s="11" t="n"/>
-      <c r="J153" s="12" t="n"/>
+      <c r="J153" s="12" t="inlineStr">
+        <is>
+          <t>Cubierta por la investigación (API_SEL_ML @TIPO 3 y 4). Revisar en Sprint Planning 6.</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="41.4" customHeight="1" s="19">
       <c r="A154" s="11" t="inlineStr">
@@ -12386,7 +12418,11 @@
         </is>
       </c>
       <c r="I154" s="11" t="n"/>
-      <c r="J154" s="12" t="n"/>
+      <c r="J154" s="12" t="inlineStr">
+        <is>
+          <t>Datos reales: versiones v1–v2 (FAILURE), v1 (RUL), v1 (VISION) registradas en Azure ML; las sintéticas marcadas en la observación.</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="27.6" customHeight="1" s="19">
       <c r="A155" s="11" t="inlineStr">
@@ -12428,7 +12464,11 @@
         </is>
       </c>
       <c r="I155" s="11" t="n"/>
-      <c r="J155" s="12" t="n"/>
+      <c r="J155" s="12" t="inlineStr">
+        <is>
+          <t>Cubierta parcialmente por SIGMA AI › Experimentos (tarjetas 2 y 3: corridas, versiones, publicar, verificar en Azure). Falta comparar versiones lado a lado (criterio 3).</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="41.4" customHeight="1" s="19">
       <c r="A156" s="11" t="inlineStr">
@@ -12466,11 +12506,17 @@
       </c>
       <c r="H156" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I156" s="11" t="n"/>
-      <c r="J156" s="12" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="I156" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J156" s="12" t="inlineStr">
+        <is>
+          <t>Investigación Azure ML: permiso ENTRENAR MODELOS en la API (ExigirPermiso) y función «Entrenar y publicar» en la web.</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="41.4" customHeight="1" s="19">
       <c r="A157" s="11" t="inlineStr">
@@ -12634,11 +12680,17 @@
       </c>
       <c r="H160" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I160" s="11" t="n"/>
-      <c r="J160" s="12" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="I160" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J160" s="12" t="inlineStr">
+        <is>
+          <t>Investigación Azure ML (BD/245–247): Dataset_Entrenamiento revisado; FNC_ML_ACTIVO_HISTORICO_V1 y FNC_ML_COMPONENTE_HISTORICO_V1 (sin fuga, con censura).</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="27.6" customHeight="1" s="19">
       <c r="A161" s="11" t="inlineStr">
@@ -12680,7 +12732,11 @@
         </is>
       </c>
       <c r="I161" s="11" t="n"/>
-      <c r="J161" s="12" t="n"/>
+      <c r="J161" s="12" t="inlineStr">
+        <is>
+          <t>Cubierta por la investigación (API_SEL_ML_DATASET_FALLA/RUL/VISION + API_INS_ML_DATASET, Bryan). Revisar en Sprint Planning 6.</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="27.6" customHeight="1" s="19">
       <c r="A162" s="11" t="inlineStr">
@@ -12722,7 +12778,11 @@
         </is>
       </c>
       <c r="I162" s="11" t="n"/>
-      <c r="J162" s="12" t="n"/>
+      <c r="J162" s="12" t="inlineStr">
+        <is>
+          <t>Cubierta por la investigación (reglas en los SP de dataset, Bryan). Revisar en Sprint Planning 6.</t>
+        </is>
+      </c>
     </row>
     <row r="163" ht="27.6" customHeight="1" s="19">
       <c r="A163" s="11" t="inlineStr">
@@ -12760,11 +12820,17 @@
       </c>
       <c r="H163" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I163" s="11" t="n"/>
-      <c r="J163" s="12" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="I163" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J163" s="12" t="inlineStr">
+        <is>
+          <t>Investigación Azure ML: API_SEL_ML @TIPO 2 (datasets) y GET /sigma-ai/datasets.</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="27.6" customHeight="1" s="19">
       <c r="A164" s="11" t="inlineStr">
@@ -12806,7 +12872,11 @@
         </is>
       </c>
       <c r="I164" s="11" t="n"/>
-      <c r="J164" s="12" t="n"/>
+      <c r="J164" s="12" t="inlineStr">
+        <is>
+          <t>Datos reales: datasets FALLA30-20260918-0120 y RUL-20260918-0449 registrados para Hamburgo.</t>
+        </is>
+      </c>
     </row>
     <row r="165" ht="27.6" customHeight="1" s="19">
       <c r="A165" s="11" t="inlineStr">
@@ -12844,11 +12914,17 @@
       </c>
       <c r="H165" s="11" t="inlineStr">
         <is>
-          <t>Por hacer</t>
-        </is>
-      </c>
-      <c r="I165" s="11" t="n"/>
-      <c r="J165" s="12" t="n"/>
+          <t>En revisión</t>
+        </is>
+      </c>
+      <c r="I165" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="J165" s="12" t="inlineStr">
+        <is>
+          <t>Investigación Azure ML: tarjeta 1 de SIGMA AI › Experimentos (ver muestra, registrar dataset con conteos y SHA-256, CSV).</t>
+        </is>
+      </c>
     </row>
     <row r="166" ht="27.6" customHeight="1" s="19">
       <c r="A166" s="11" t="inlineStr">

</xml_diff>